<commit_message>
rerun to include 2025
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="207">
   <si>
     <t>TileID</t>
   </si>
@@ -127,12 +127,18 @@
     <t>Franklin</t>
   </si>
   <si>
+    <t>Prairie</t>
+  </si>
+  <si>
     <t>Bellefontaine</t>
   </si>
   <si>
     <t>Bexley</t>
   </si>
   <si>
+    <t>Etna</t>
+  </si>
+  <si>
     <t>Canal Winchester</t>
   </si>
   <si>
@@ -175,15 +181,9 @@
     <t>Heath</t>
   </si>
   <si>
-    <t>Hebron</t>
-  </si>
-  <si>
     <t>Hilliard</t>
   </si>
   <si>
-    <t>Johnstown</t>
-  </si>
-  <si>
     <t>Lancaster</t>
   </si>
   <si>
@@ -208,22 +208,25 @@
     <t>Newark</t>
   </si>
   <si>
+    <t>New Lexington</t>
+  </si>
+  <si>
     <t>Obetz</t>
   </si>
   <si>
-    <t>Pataskala</t>
-  </si>
-  <si>
     <t>Pickerington</t>
   </si>
   <si>
+    <t>Plain City</t>
+  </si>
+  <si>
     <t>Powell</t>
   </si>
   <si>
     <t>Reynoldsburg</t>
   </si>
   <si>
-    <t>Somerset</t>
+    <t>South Bloomfield</t>
   </si>
   <si>
     <t>Sunbury</t>
@@ -232,6 +235,9 @@
     <t>Upper Arlington</t>
   </si>
   <si>
+    <t>Urbancrest</t>
+  </si>
+  <si>
     <t>Westerville</t>
   </si>
   <si>
@@ -310,12 +316,18 @@
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US390492828099999.svg</t>
   </si>
   <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US390496457099999.svg</t>
+  </si>
+  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3905130.svg</t>
   </si>
   <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3906278.svg</t>
   </si>
   <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US390892569099999.svg</t>
+  </si>
+  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3911332.svg</t>
   </si>
   <si>
@@ -358,15 +370,9 @@
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3934748.svg</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3934790.svg</t>
-  </si>
-  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3935476.svg</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3939340.svg</t>
-  </si>
-  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3941720.svg</t>
   </si>
   <si>
@@ -391,22 +397,25 @@
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3954040.svg</t>
   </si>
   <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3954866.svg</t>
+  </si>
+  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3957862.svg</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3961112.svg</t>
-  </si>
-  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3962498.svg</t>
   </si>
   <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3963030.svg</t>
+  </si>
+  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3964486.svg</t>
   </si>
   <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3966390.svg</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3972977.svg</t>
+    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3973068.svg</t>
   </si>
   <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3975602.svg</t>
@@ -415,6 +424,9 @@
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3979002.svg</t>
   </si>
   <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3979100.svg</t>
+  </si>
+  <si>
     <t>https://raw.githubusercontent.com/morpc-insights/altfuelstations/refs/heads/main/output_data/charts/M100000US3983342.svg</t>
   </si>
   <si>
@@ -499,12 +511,18 @@
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US390492828099999</t>
   </si>
   <si>
+    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US390496457099999</t>
+  </si>
+  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3905130</t>
   </si>
   <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3906278</t>
   </si>
   <si>
+    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US390892569099999</t>
+  </si>
+  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3911332</t>
   </si>
   <si>
@@ -547,15 +565,9 @@
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3934748</t>
   </si>
   <si>
-    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3934790</t>
-  </si>
-  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3935476</t>
   </si>
   <si>
-    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3939340</t>
-  </si>
-  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3941720</t>
   </si>
   <si>
@@ -580,28 +592,34 @@
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3954040</t>
   </si>
   <si>
+    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3954866</t>
+  </si>
+  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3957862</t>
   </si>
   <si>
-    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3961112</t>
-  </si>
-  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3962498</t>
   </si>
   <si>
+    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3963030</t>
+  </si>
+  <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3964486</t>
   </si>
   <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3966390</t>
   </si>
   <si>
-    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3972977</t>
+    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3973068</t>
   </si>
   <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3975602</t>
   </si>
   <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3979002</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3979100</t>
   </si>
   <si>
     <t>https://www.arcgis.com/apps/dashboards/87fd6a0b569b430c9e4c6e7fa4fbd4c5#geoid=M100000US3983342</t>
@@ -987,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -1042,28 +1060,28 @@
         <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K2" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1074,28 +1092,28 @@
         <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J3" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1106,28 +1124,28 @@
         <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1138,28 +1156,28 @@
         <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1170,28 +1188,28 @@
         <v>20</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J6" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K6" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1202,28 +1220,28 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1234,28 +1252,28 @@
         <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I8" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J8" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K8" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -1266,28 +1284,28 @@
         <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I9" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J9" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K9" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -1298,28 +1316,28 @@
         <v>24</v>
       </c>
       <c r="F10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -1330,28 +1348,28 @@
         <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I11" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J11" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K11" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1362,28 +1380,28 @@
         <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J12" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K12" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1394,28 +1412,28 @@
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I13" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J13" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K13" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1426,28 +1444,28 @@
         <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K14" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -1458,28 +1476,28 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I15" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J15" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K15" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -1490,28 +1508,28 @@
         <v>30</v>
       </c>
       <c r="F16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I16" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J16" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K16" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17" spans="3:14">
@@ -1522,28 +1540,28 @@
         <v>31</v>
       </c>
       <c r="F17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I17" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J17" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K17" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="3:14">
@@ -1551,28 +1569,28 @@
         <v>32</v>
       </c>
       <c r="F18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I18" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J18" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K18" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="19" spans="3:14">
@@ -1580,28 +1598,28 @@
         <v>33</v>
       </c>
       <c r="F19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I19" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J19" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K19" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" spans="3:14">
@@ -1609,28 +1627,28 @@
         <v>34</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I20" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J20" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K20" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="21" spans="3:14">
@@ -1638,28 +1656,28 @@
         <v>35</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I21" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J21" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K21" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="3:14">
@@ -1667,28 +1685,28 @@
         <v>36</v>
       </c>
       <c r="F22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I22" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J22" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K22" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="23" spans="3:14">
@@ -1696,28 +1714,28 @@
         <v>37</v>
       </c>
       <c r="F23" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G23" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I23" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J23" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K23" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="3:14">
@@ -1725,28 +1743,28 @@
         <v>38</v>
       </c>
       <c r="F24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I24" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J24" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K24" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" spans="3:14">
@@ -1754,28 +1772,28 @@
         <v>39</v>
       </c>
       <c r="F25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I25" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J25" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K25" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="26" spans="3:14">
@@ -1783,28 +1801,28 @@
         <v>40</v>
       </c>
       <c r="F26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I26" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J26" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K26" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" spans="3:14">
@@ -1812,28 +1830,28 @@
         <v>41</v>
       </c>
       <c r="F27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I27" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J27" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K27" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="28" spans="3:14">
@@ -1841,28 +1859,28 @@
         <v>42</v>
       </c>
       <c r="F28" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G28" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I28" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J28" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K28" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="29" spans="3:14">
@@ -1870,28 +1888,28 @@
         <v>43</v>
       </c>
       <c r="F29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I29" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J29" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K29" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="30" spans="3:14">
@@ -1899,28 +1917,28 @@
         <v>44</v>
       </c>
       <c r="F30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I30" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J30" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K30" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="31" spans="3:14">
@@ -1928,28 +1946,28 @@
         <v>45</v>
       </c>
       <c r="F31" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G31" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I31" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J31" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K31" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32" spans="3:14">
@@ -1957,28 +1975,28 @@
         <v>46</v>
       </c>
       <c r="F32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I32" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J32" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K32" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" spans="4:14">
@@ -1986,28 +2004,28 @@
         <v>47</v>
       </c>
       <c r="F33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I33" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J33" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K33" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="4:14">
@@ -2015,28 +2033,28 @@
         <v>48</v>
       </c>
       <c r="F34" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G34" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I34" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J34" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K34" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35" spans="4:14">
@@ -2044,28 +2062,28 @@
         <v>49</v>
       </c>
       <c r="F35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I35" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J35" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K35" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="36" spans="4:14">
@@ -2073,28 +2091,28 @@
         <v>50</v>
       </c>
       <c r="F36" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G36" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I36" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J36" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K36" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="37" spans="4:14">
@@ -2102,28 +2120,28 @@
         <v>51</v>
       </c>
       <c r="F37" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G37" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I37" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J37" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K37" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="38" spans="4:14">
@@ -2131,28 +2149,28 @@
         <v>52</v>
       </c>
       <c r="F38" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G38" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I38" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J38" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K38" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="39" spans="4:14">
@@ -2160,28 +2178,28 @@
         <v>53</v>
       </c>
       <c r="F39" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G39" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I39" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J39" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K39" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="40" spans="4:14">
@@ -2189,28 +2207,28 @@
         <v>54</v>
       </c>
       <c r="F40" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G40" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I40" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J40" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K40" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" spans="4:14">
@@ -2218,28 +2236,28 @@
         <v>55</v>
       </c>
       <c r="F41" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G41" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I41" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J41" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K41" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="42" spans="4:14">
@@ -2247,28 +2265,28 @@
         <v>56</v>
       </c>
       <c r="F42" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G42" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I42" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J42" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K42" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" spans="4:14">
@@ -2276,28 +2294,28 @@
         <v>57</v>
       </c>
       <c r="F43" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G43" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I43" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J43" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K43" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44" spans="4:14">
@@ -2305,28 +2323,28 @@
         <v>58</v>
       </c>
       <c r="F44" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G44" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I44" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J44" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K44" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="45" spans="4:14">
@@ -2334,28 +2352,28 @@
         <v>59</v>
       </c>
       <c r="F45" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G45" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I45" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J45" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K45" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="46" spans="4:14">
@@ -2363,28 +2381,28 @@
         <v>60</v>
       </c>
       <c r="F46" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G46" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I46" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J46" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K46" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" spans="4:14">
@@ -2392,28 +2410,28 @@
         <v>61</v>
       </c>
       <c r="F47" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G47" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I47" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J47" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K47" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="48" spans="4:14">
@@ -2421,28 +2439,28 @@
         <v>62</v>
       </c>
       <c r="F48" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G48" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I48" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J48" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K48" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="49" spans="4:14">
@@ -2450,28 +2468,28 @@
         <v>63</v>
       </c>
       <c r="F49" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G49" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I49" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J49" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K49" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="50" spans="4:14">
@@ -2479,28 +2497,28 @@
         <v>64</v>
       </c>
       <c r="F50" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G50" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I50" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J50" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K50" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="51" spans="4:14">
@@ -2508,28 +2526,28 @@
         <v>65</v>
       </c>
       <c r="F51" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G51" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I51" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J51" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K51" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" spans="4:14">
@@ -2537,28 +2555,28 @@
         <v>66</v>
       </c>
       <c r="F52" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G52" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I52" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J52" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K52" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="53" spans="4:14">
@@ -2566,28 +2584,28 @@
         <v>67</v>
       </c>
       <c r="F53" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G53" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J53" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K53" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="54" spans="4:14">
@@ -2595,28 +2613,28 @@
         <v>68</v>
       </c>
       <c r="F54" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G54" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I54" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J54" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K54" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" spans="4:14">
@@ -2624,28 +2642,28 @@
         <v>69</v>
       </c>
       <c r="F55" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G55" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I55" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J55" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K55" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="56" spans="4:14">
@@ -2653,28 +2671,28 @@
         <v>70</v>
       </c>
       <c r="F56" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G56" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I56" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J56" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K56" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="57" spans="4:14">
@@ -2682,28 +2700,28 @@
         <v>71</v>
       </c>
       <c r="F57" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G57" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I57" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J57" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K57" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="58" spans="4:14">
@@ -2711,28 +2729,28 @@
         <v>72</v>
       </c>
       <c r="F58" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G58" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I58" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J58" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K58" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="59" spans="4:14">
@@ -2740,28 +2758,28 @@
         <v>73</v>
       </c>
       <c r="F59" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G59" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I59" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J59" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K59" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="60" spans="4:14">
@@ -2769,28 +2787,28 @@
         <v>74</v>
       </c>
       <c r="F60" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G60" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I60" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J60" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K60" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="61" spans="4:14">
@@ -2798,28 +2816,86 @@
         <v>75</v>
       </c>
       <c r="F61" t="s">
+        <v>78</v>
+      </c>
+      <c r="G61" t="s">
+        <v>78</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I61" t="s">
+        <v>141</v>
+      </c>
+      <c r="J61" t="s">
+        <v>142</v>
+      </c>
+      <c r="K61" t="s">
+        <v>143</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="62" spans="4:14">
+      <c r="D62" t="s">
         <v>76</v>
       </c>
-      <c r="G61" t="s">
-        <v>76</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="I61" t="s">
-        <v>137</v>
-      </c>
-      <c r="J61" t="s">
-        <v>138</v>
-      </c>
-      <c r="K61" t="s">
+      <c r="F62" t="s">
+        <v>78</v>
+      </c>
+      <c r="G62" t="s">
+        <v>78</v>
+      </c>
+      <c r="H62" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="M61" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="N61" s="2" t="s">
-        <v>200</v>
+      <c r="I62" t="s">
+        <v>141</v>
+      </c>
+      <c r="J62" t="s">
+        <v>142</v>
+      </c>
+      <c r="K62" t="s">
+        <v>143</v>
+      </c>
+      <c r="M62" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="N62" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="63" spans="4:14">
+      <c r="D63" t="s">
+        <v>77</v>
+      </c>
+      <c r="F63" t="s">
+        <v>78</v>
+      </c>
+      <c r="G63" t="s">
+        <v>78</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I63" t="s">
+        <v>141</v>
+      </c>
+      <c r="J63" t="s">
+        <v>142</v>
+      </c>
+      <c r="K63" t="s">
+        <v>143</v>
+      </c>
+      <c r="M63" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="N63" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -2888,61 +2964,61 @@
     <hyperlink ref="M22" r:id="rId62" location="geoid=M100000US390492828099999"/>
     <hyperlink ref="N22" r:id="rId63"/>
     <hyperlink ref="H23" r:id="rId64"/>
-    <hyperlink ref="M23" r:id="rId65" location="geoid=M100000US3905130"/>
+    <hyperlink ref="M23" r:id="rId65" location="geoid=M100000US390496457099999"/>
     <hyperlink ref="N23" r:id="rId66"/>
     <hyperlink ref="H24" r:id="rId67"/>
-    <hyperlink ref="M24" r:id="rId68" location="geoid=M100000US3906278"/>
+    <hyperlink ref="M24" r:id="rId68" location="geoid=M100000US3905130"/>
     <hyperlink ref="N24" r:id="rId69"/>
     <hyperlink ref="H25" r:id="rId70"/>
-    <hyperlink ref="M25" r:id="rId71" location="geoid=M100000US3911332"/>
+    <hyperlink ref="M25" r:id="rId71" location="geoid=M100000US3906278"/>
     <hyperlink ref="N25" r:id="rId72"/>
     <hyperlink ref="H26" r:id="rId73"/>
-    <hyperlink ref="M26" r:id="rId74" location="geoid=M100000US3914184"/>
+    <hyperlink ref="M26" r:id="rId74" location="geoid=M100000US390892569099999"/>
     <hyperlink ref="N26" r:id="rId75"/>
     <hyperlink ref="H27" r:id="rId76"/>
-    <hyperlink ref="M27" r:id="rId77" location="geoid=M100000US3915070"/>
+    <hyperlink ref="M27" r:id="rId77" location="geoid=M100000US3911332"/>
     <hyperlink ref="N27" r:id="rId78"/>
     <hyperlink ref="H28" r:id="rId79"/>
-    <hyperlink ref="M28" r:id="rId80" location="geoid=M100000US391593904699999"/>
+    <hyperlink ref="M28" r:id="rId80" location="geoid=M100000US3914184"/>
     <hyperlink ref="N28" r:id="rId81"/>
     <hyperlink ref="H29" r:id="rId82"/>
-    <hyperlink ref="M29" r:id="rId83" location="geoid=M100000US3918000"/>
+    <hyperlink ref="M29" r:id="rId83" location="geoid=M100000US3915070"/>
     <hyperlink ref="N29" r:id="rId84"/>
     <hyperlink ref="H30" r:id="rId85"/>
-    <hyperlink ref="M30" r:id="rId86" location="geoid=M100000US3921434"/>
+    <hyperlink ref="M30" r:id="rId86" location="geoid=M100000US391593904699999"/>
     <hyperlink ref="N30" r:id="rId87"/>
     <hyperlink ref="H31" r:id="rId88"/>
-    <hyperlink ref="M31" r:id="rId89" location="geoid=M100000US3922694"/>
+    <hyperlink ref="M31" r:id="rId89" location="geoid=M100000US3918000"/>
     <hyperlink ref="N31" r:id="rId90"/>
     <hyperlink ref="H32" r:id="rId91"/>
-    <hyperlink ref="M32" r:id="rId92" location="geoid=M100000US3929106"/>
+    <hyperlink ref="M32" r:id="rId92" location="geoid=M100000US3921434"/>
     <hyperlink ref="N32" r:id="rId93"/>
     <hyperlink ref="H33" r:id="rId94"/>
-    <hyperlink ref="M33" r:id="rId95" location="geoid=M100000US3929246"/>
+    <hyperlink ref="M33" r:id="rId95" location="geoid=M100000US3922694"/>
     <hyperlink ref="N33" r:id="rId96"/>
     <hyperlink ref="H34" r:id="rId97"/>
-    <hyperlink ref="M34" r:id="rId98" location="geoid=M100000US3931304"/>
+    <hyperlink ref="M34" r:id="rId98" location="geoid=M100000US3929106"/>
     <hyperlink ref="N34" r:id="rId99"/>
     <hyperlink ref="H35" r:id="rId100"/>
-    <hyperlink ref="M35" r:id="rId101" location="geoid=M100000US3931402"/>
+    <hyperlink ref="M35" r:id="rId101" location="geoid=M100000US3929246"/>
     <hyperlink ref="N35" r:id="rId102"/>
     <hyperlink ref="H36" r:id="rId103"/>
-    <hyperlink ref="M36" r:id="rId104" location="geoid=M100000US3932592"/>
+    <hyperlink ref="M36" r:id="rId104" location="geoid=M100000US3931304"/>
     <hyperlink ref="N36" r:id="rId105"/>
     <hyperlink ref="H37" r:id="rId106"/>
-    <hyperlink ref="M37" r:id="rId107" location="geoid=M100000US3932606"/>
+    <hyperlink ref="M37" r:id="rId107" location="geoid=M100000US3931402"/>
     <hyperlink ref="N37" r:id="rId108"/>
     <hyperlink ref="H38" r:id="rId109"/>
-    <hyperlink ref="M38" r:id="rId110" location="geoid=M100000US3934748"/>
+    <hyperlink ref="M38" r:id="rId110" location="geoid=M100000US3932592"/>
     <hyperlink ref="N38" r:id="rId111"/>
     <hyperlink ref="H39" r:id="rId112"/>
-    <hyperlink ref="M39" r:id="rId113" location="geoid=M100000US3934790"/>
+    <hyperlink ref="M39" r:id="rId113" location="geoid=M100000US3932606"/>
     <hyperlink ref="N39" r:id="rId114"/>
     <hyperlink ref="H40" r:id="rId115"/>
-    <hyperlink ref="M40" r:id="rId116" location="geoid=M100000US3935476"/>
+    <hyperlink ref="M40" r:id="rId116" location="geoid=M100000US3934748"/>
     <hyperlink ref="N40" r:id="rId117"/>
     <hyperlink ref="H41" r:id="rId118"/>
-    <hyperlink ref="M41" r:id="rId119" location="geoid=M100000US3939340"/>
+    <hyperlink ref="M41" r:id="rId119" location="geoid=M100000US3935476"/>
     <hyperlink ref="N41" r:id="rId120"/>
     <hyperlink ref="H42" r:id="rId121"/>
     <hyperlink ref="M42" r:id="rId122" location="geoid=M100000US3941720"/>
@@ -2969,41 +3045,47 @@
     <hyperlink ref="M49" r:id="rId143" location="geoid=M100000US3954040"/>
     <hyperlink ref="N49" r:id="rId144"/>
     <hyperlink ref="H50" r:id="rId145"/>
-    <hyperlink ref="M50" r:id="rId146" location="geoid=M100000US3957862"/>
+    <hyperlink ref="M50" r:id="rId146" location="geoid=M100000US3954866"/>
     <hyperlink ref="N50" r:id="rId147"/>
     <hyperlink ref="H51" r:id="rId148"/>
-    <hyperlink ref="M51" r:id="rId149" location="geoid=M100000US3961112"/>
+    <hyperlink ref="M51" r:id="rId149" location="geoid=M100000US3957862"/>
     <hyperlink ref="N51" r:id="rId150"/>
     <hyperlink ref="H52" r:id="rId151"/>
     <hyperlink ref="M52" r:id="rId152" location="geoid=M100000US3962498"/>
     <hyperlink ref="N52" r:id="rId153"/>
     <hyperlink ref="H53" r:id="rId154"/>
-    <hyperlink ref="M53" r:id="rId155" location="geoid=M100000US3964486"/>
+    <hyperlink ref="M53" r:id="rId155" location="geoid=M100000US3963030"/>
     <hyperlink ref="N53" r:id="rId156"/>
     <hyperlink ref="H54" r:id="rId157"/>
-    <hyperlink ref="M54" r:id="rId158" location="geoid=M100000US3966390"/>
+    <hyperlink ref="M54" r:id="rId158" location="geoid=M100000US3964486"/>
     <hyperlink ref="N54" r:id="rId159"/>
     <hyperlink ref="H55" r:id="rId160"/>
-    <hyperlink ref="M55" r:id="rId161" location="geoid=M100000US3972977"/>
+    <hyperlink ref="M55" r:id="rId161" location="geoid=M100000US3966390"/>
     <hyperlink ref="N55" r:id="rId162"/>
     <hyperlink ref="H56" r:id="rId163"/>
-    <hyperlink ref="M56" r:id="rId164" location="geoid=M100000US3975602"/>
+    <hyperlink ref="M56" r:id="rId164" location="geoid=M100000US3973068"/>
     <hyperlink ref="N56" r:id="rId165"/>
     <hyperlink ref="H57" r:id="rId166"/>
-    <hyperlink ref="M57" r:id="rId167" location="geoid=M100000US3979002"/>
+    <hyperlink ref="M57" r:id="rId167" location="geoid=M100000US3975602"/>
     <hyperlink ref="N57" r:id="rId168"/>
     <hyperlink ref="H58" r:id="rId169"/>
-    <hyperlink ref="M58" r:id="rId170" location="geoid=M100000US3983342"/>
+    <hyperlink ref="M58" r:id="rId170" location="geoid=M100000US3979002"/>
     <hyperlink ref="N58" r:id="rId171"/>
     <hyperlink ref="H59" r:id="rId172"/>
-    <hyperlink ref="M59" r:id="rId173" location="geoid=M100000US3983580"/>
+    <hyperlink ref="M59" r:id="rId173" location="geoid=M100000US3979100"/>
     <hyperlink ref="N59" r:id="rId174"/>
     <hyperlink ref="H60" r:id="rId175"/>
-    <hyperlink ref="M60" r:id="rId176" location="geoid=M100000US3984742"/>
+    <hyperlink ref="M60" r:id="rId176" location="geoid=M100000US3983342"/>
     <hyperlink ref="N60" r:id="rId177"/>
     <hyperlink ref="H61" r:id="rId178"/>
-    <hyperlink ref="M61" r:id="rId179" location="geoid=M100000US3986604"/>
+    <hyperlink ref="M61" r:id="rId179" location="geoid=M100000US3983580"/>
     <hyperlink ref="N61" r:id="rId180"/>
+    <hyperlink ref="H62" r:id="rId181"/>
+    <hyperlink ref="M62" r:id="rId182" location="geoid=M100000US3984742"/>
+    <hyperlink ref="N62" r:id="rId183"/>
+    <hyperlink ref="H63" r:id="rId184"/>
+    <hyperlink ref="M63" r:id="rId185" location="geoid=M100000US3986604"/>
+    <hyperlink ref="N63" r:id="rId186"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>